<commit_message>
feat: Add join queries and company table with sample data
Enhanced `JOINS.sql` with Full, Left, Right, and Cross Join examples.
Modified `empj` table query and added Cartesian product examples.
Updated `differences of joins.xlsx` with all the JOINS differences and their definitions.
Created `company` table in `company table creation.sql` with columns
`cid`, `company_name`, `location`, and `count`. Added `BULK INSERT`
to load data from `company.csv` and verified with a `SELECT` query.
Included `company.csv` with 15 rows of sample data.
</commit_message>
<xml_diff>
--- a/differences of joins.xlsx
+++ b/differences of joins.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQL-Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9AF97C6-536C-418F-8CB6-8CCC526AE495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A97F16-5630-4C39-A534-AB9CBCC4009F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3741AAEB-0694-418D-9DFA-6921BDB9A86A}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="16">
   <si>
     <t>employee</t>
   </si>
@@ -51,6 +51,39 @@
   <si>
     <t>NULL</t>
   </si>
+  <si>
+    <t>inner join</t>
+  </si>
+  <si>
+    <t>full join</t>
+  </si>
+  <si>
+    <t>give all data from the table even if there is no data it will print null</t>
+  </si>
+  <si>
+    <t>combines both tables common values</t>
+  </si>
+  <si>
+    <t>left join</t>
+  </si>
+  <si>
+    <t>get all data from left table &amp; common data from right table and others set to null</t>
+  </si>
+  <si>
+    <t>right join</t>
+  </si>
+  <si>
+    <t>get all data from right table &amp; common data from left table and others set to null</t>
+  </si>
+  <si>
+    <t>Raw Data</t>
+  </si>
+  <si>
+    <t>cross join</t>
+  </si>
+  <si>
+    <t>every record of one table is joined with every record of another table</t>
+  </si>
 </sst>
 </file>
 
@@ -65,7 +98,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -81,6 +114,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -112,12 +151,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -126,7 +171,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -443,435 +491,727 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276BCC7F-CE80-48BA-BCF9-904138AD6C32}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr defaultColWidth="14.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="14.5546875" style="1"/>
-    <col min="4" max="5" width="26.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" style="1"/>
-    <col min="7" max="8" width="29.77734375" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="14.5546875" style="1"/>
+    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="5.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.77734375" style="1" customWidth="1"/>
+    <col min="7" max="8" width="5.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="4.77734375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="6.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="6" style="1" customWidth="1"/>
+    <col min="13" max="13" width="5.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.6640625" style="1" customWidth="1"/>
+    <col min="15" max="16" width="14.5546875" style="1"/>
+    <col min="17" max="17" width="68" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="14.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="G2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="6"/>
+      <c r="M2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="6"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2">
+        <v>2</v>
+      </c>
+      <c r="J4" s="2">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2">
+        <v>2</v>
+      </c>
+      <c r="M4" s="2">
+        <v>2</v>
+      </c>
+      <c r="N4" s="2">
+        <v>2</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="H1" s="3"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2">
-        <v>2</v>
-      </c>
-      <c r="E3" s="2">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="B5" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="D5" s="2">
         <v>3</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E5" s="2">
         <v>3</v>
       </c>
-      <c r="E4" s="2">
+      <c r="G5" s="2">
         <v>3</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H5" s="2">
         <v>3</v>
       </c>
-      <c r="H4" s="2">
+      <c r="J5" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2">
-        <v>4</v>
-      </c>
-      <c r="D5" s="2">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4</v>
-      </c>
-      <c r="G5" s="2">
-        <v>4</v>
-      </c>
-      <c r="H5" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="K5" s="2">
+        <v>3</v>
+      </c>
+      <c r="M5" s="2">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2">
+        <v>3</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H6" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="J6" s="2">
+        <v>4</v>
+      </c>
+      <c r="K6" s="2">
+        <v>4</v>
+      </c>
+      <c r="M6" s="2">
+        <v>4</v>
+      </c>
+      <c r="N6" s="2">
+        <v>4</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H7" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="J7" s="2">
+        <v>5</v>
+      </c>
+      <c r="K7" s="2">
+        <v>5</v>
+      </c>
+      <c r="M7" s="2">
+        <v>5</v>
+      </c>
+      <c r="N7" s="2">
+        <v>5</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <v>6</v>
+      </c>
+      <c r="D8" s="2">
+        <v>6</v>
+      </c>
+      <c r="E8" s="2">
+        <v>6</v>
+      </c>
+      <c r="G8" s="2">
+        <v>6</v>
+      </c>
+      <c r="H8" s="2">
+        <v>6</v>
+      </c>
+      <c r="J8" s="2">
+        <v>6</v>
+      </c>
+      <c r="K8" s="2">
+        <v>6</v>
+      </c>
+      <c r="M8" s="2">
+        <v>6</v>
+      </c>
+      <c r="N8" s="2">
+        <v>6</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q8" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B9" s="2">
         <v>7</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D9" s="2">
         <v>7</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E9" s="2">
         <v>7</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G9" s="2">
         <v>7</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H9" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="J9" s="2">
+        <v>7</v>
+      </c>
+      <c r="K9" s="2">
+        <v>7</v>
+      </c>
+      <c r="M9" s="2">
+        <v>7</v>
+      </c>
+      <c r="N9" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B10" s="2">
         <v>8</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D10" s="2">
         <v>8</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E10" s="2">
         <v>8</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G10" s="2">
         <v>8</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H10" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2">
-        <v>9</v>
-      </c>
-      <c r="E10" s="2">
-        <v>9</v>
-      </c>
-      <c r="G10" s="2">
-        <v>9</v>
-      </c>
-      <c r="H10" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J10" s="2">
+        <v>8</v>
+      </c>
+      <c r="K10" s="2">
+        <v>8</v>
+      </c>
+      <c r="M10" s="2">
+        <v>8</v>
+      </c>
+      <c r="N10" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2">
+        <v>9</v>
+      </c>
+      <c r="D11" s="2">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2">
+        <v>9</v>
+      </c>
+      <c r="G11" s="2">
+        <v>9</v>
+      </c>
+      <c r="H11" s="2">
+        <v>9</v>
+      </c>
+      <c r="J11" s="2">
+        <v>9</v>
+      </c>
+      <c r="K11" s="2">
+        <v>9</v>
+      </c>
+      <c r="M11" s="2">
+        <v>9</v>
+      </c>
+      <c r="N11" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B12" s="2">
         <v>10</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D12" s="2">
         <v>10</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E12" s="2">
         <v>10</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G12" s="2">
         <v>10</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H12" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2">
-        <v>11</v>
-      </c>
-      <c r="E12" s="2">
-        <v>11</v>
-      </c>
-      <c r="G12" s="2">
-        <v>11</v>
-      </c>
-      <c r="H12" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J12" s="2">
+        <v>10</v>
+      </c>
+      <c r="K12" s="2">
+        <v>10</v>
+      </c>
+      <c r="M12" s="2">
+        <v>10</v>
+      </c>
+      <c r="N12" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <v>11</v>
+      </c>
+      <c r="D13" s="2">
+        <v>11</v>
+      </c>
+      <c r="E13" s="2">
+        <v>11</v>
+      </c>
+      <c r="G13" s="2">
+        <v>11</v>
+      </c>
+      <c r="H13" s="2">
+        <v>11</v>
+      </c>
+      <c r="J13" s="2">
+        <v>11</v>
+      </c>
+      <c r="K13" s="2">
+        <v>11</v>
+      </c>
+      <c r="M13" s="2">
+        <v>11</v>
+      </c>
+      <c r="N13" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B14" s="2">
         <v>12</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D14" s="2">
         <v>12</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E14" s="2">
         <v>12</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G14" s="2">
         <v>12</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H14" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="J14" s="2">
+        <v>12</v>
+      </c>
+      <c r="K14" s="2">
+        <v>12</v>
+      </c>
+      <c r="M14" s="2">
+        <v>12</v>
+      </c>
+      <c r="N14" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B15" s="2">
         <v>13</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D15" s="2">
         <v>13</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E15" s="2">
         <v>13</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G15" s="2">
         <v>13</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H15" s="2">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
+      <c r="J15" s="2">
+        <v>13</v>
+      </c>
+      <c r="K15" s="2">
+        <v>13</v>
+      </c>
+      <c r="M15" s="2">
+        <v>13</v>
+      </c>
+      <c r="N15" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B16" s="2">
         <v>14</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D16" s="2">
         <v>14</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E16" s="2">
         <v>14</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G16" s="2">
         <v>14</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H16" s="2">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
+      <c r="J16" s="2">
+        <v>14</v>
+      </c>
+      <c r="K16" s="2">
+        <v>14</v>
+      </c>
+      <c r="M16" s="2">
+        <v>14</v>
+      </c>
+      <c r="N16" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B17" s="2">
         <v>15</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D17" s="2">
         <v>15</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E17" s="2">
         <v>15</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G17" s="2">
         <v>15</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H17" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+      <c r="J17" s="2">
+        <v>15</v>
+      </c>
+      <c r="K17" s="2">
+        <v>15</v>
+      </c>
+      <c r="M17" s="2">
+        <v>15</v>
+      </c>
+      <c r="N17" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B18" s="2">
         <v>30</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G18" s="2">
         <v>16</v>
       </c>
-      <c r="H17" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="H18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J18" s="2">
+        <v>16</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B19" s="2">
         <v>31</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G19" s="2">
         <v>17</v>
       </c>
-      <c r="H18" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
+      <c r="H19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J19" s="2">
+        <v>17</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B20" s="2">
         <v>32</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G20" s="2">
         <v>18</v>
       </c>
-      <c r="H19" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
+      <c r="H20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J20" s="2">
+        <v>18</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B21" s="2">
         <v>33</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G21" s="2">
         <v>19</v>
       </c>
-      <c r="H20" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
+      <c r="H21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J21" s="2">
+        <v>19</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
         <v>20</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G22" s="2">
         <v>20</v>
       </c>
-      <c r="H21" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G22" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H22" s="2">
+      <c r="H22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J22" s="2">
+        <v>20</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H23" s="2">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G23" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H23" s="2">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H24" s="2">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G24" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H24" s="2">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H25" s="2">
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G25" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H25" s="2">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H26" s="2">
         <v>33</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
+  <mergeCells count="5">
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -891,20 +1231,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="E1" s="5"/>
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
@@ -1216,7 +1556,7 @@
       <c r="G17" s="2">
         <v>16</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1230,7 +1570,7 @@
       <c r="G18" s="2">
         <v>17</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1244,7 +1584,7 @@
       <c r="G19" s="2">
         <v>18</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1258,7 +1598,7 @@
       <c r="G20" s="2">
         <v>19</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1269,12 +1609,12 @@
       <c r="G21" s="2">
         <v>20</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="H21" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G22" s="5" t="s">
+      <c r="G22" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H22" s="2">
@@ -1282,7 +1622,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G23" s="5" t="s">
+      <c r="G23" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H23" s="2">
@@ -1290,7 +1630,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G24" s="5" t="s">
+      <c r="G24" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H24" s="2">
@@ -1298,7 +1638,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="4" t="s">
         <v>4</v>
       </c>
       <c r="H25" s="2">

</xml_diff>